<commit_message>
Project Example 1 - Bank Rating1 is saved.
</commit_message>
<xml_diff>
--- a/test/Example 1 - Bank Rating1/Bank Rating.xlsx
+++ b/test/Example 1 - Bank Rating1/Bank Rating.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="693">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="705">
   <si>
     <t xml:space="preserve">www.commerzbank.com</t>
   </si>
@@ -4374,6 +4374,42 @@
   </si>
   <si>
     <t xml:space="preserve">SPD</t>
+  </si>
+  <si>
+    <t>Quick Liquidity Dynamic Score D2 234</t>
+  </si>
+  <si>
+    <t>Datatype myTqble extends Bank</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Default</t>
+  </si>
+  <si>
+    <t>Mandatory</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>String</t>
+  </si>
+  <si>
+    <t>field1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My тест cegth gjkt </t>
+  </si>
+  <si>
+    <t>123</t>
   </si>
 </sst>
 </file>
@@ -5622,47 +5658,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="25">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+  <cellStyleXfs count="4">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true" xfId="0">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true" xfId="1">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true" xfId="2">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false" xfId="3">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
@@ -5675,7 +5684,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5683,7 +5692,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="24" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="3" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5723,7 +5732,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5739,7 +5748,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5791,7 +5800,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6403,7 +6412,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="102" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="102" xfId="1" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6463,7 +6472,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="13" borderId="29" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="13" borderId="29" xfId="2" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6495,23 +6504,16 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="13" borderId="67" xfId="22" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="13" borderId="67" xfId="2" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="11">
+  <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Normal 7" xfId="21"/>
-    <cellStyle name="Normal_EPLI rater" xfId="22"/>
-    <cellStyle name="Обычный 2" xfId="23"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
-    <cellStyle name="Excel Built-in Heading 1" xfId="24"/>
+    <cellStyle name="Normal_EPLI rater" xfId="2"/>
+    <cellStyle name="*unknown*" xfId="1" builtinId="8"/>
+    <cellStyle name="Excel Built-in Heading 1" xfId="3"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -6652,19 +6654,19 @@
     <tabColor rgb="FF558ED5"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:J96"/>
+  <dimension ref="B1:J100"/>
   <sheetFormatPr defaultColWidth="9.09375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="9.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="42.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="76.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="5.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="24.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="19.11"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="12" style="1" width="9.11"/>
+    <col min="1" max="2" customWidth="false" hidden="false" style="1" width="9.11" collapsed="false" outlineLevel="0"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="1" width="8.56" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="1" width="16.56" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="1" width="25.66" collapsed="false" outlineLevel="0"/>
+    <col min="6" max="6" customWidth="true" hidden="false" style="1" width="42.34" collapsed="false" outlineLevel="0"/>
+    <col min="7" max="7" customWidth="true" hidden="false" style="1" width="76.67" collapsed="false" outlineLevel="0"/>
+    <col min="8" max="9" customWidth="true" hidden="false" style="1" width="5.88" collapsed="false" outlineLevel="0"/>
+    <col min="10" max="10" customWidth="true" hidden="false" style="1" width="24.99" collapsed="false" outlineLevel="0"/>
+    <col min="11" max="11" customWidth="true" hidden="false" style="1" width="19.11" collapsed="false" outlineLevel="0"/>
+    <col min="12" max="1024" customWidth="false" hidden="false" style="1" width="9.11" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7240,7 +7242,7 @@
       </c>
       <c r="E60" s="32"/>
       <c r="F60" s="33" t="s">
-        <v>119</v>
+        <v>693</v>
       </c>
       <c r="G60" s="34" t="s">
         <v>120</v>
@@ -7568,8 +7570,56 @@
         <v>179</v>
       </c>
     </row>
+    <row r="98">
+      <c r="B98" t="s" s="1">
+        <v>694</v>
+      </c>
+      <c r="C98" s="1"/>
+      <c r="D98" s="1"/>
+      <c r="E98" s="1"/>
+      <c r="F98" s="1"/>
+      <c r="G98" s="1"/>
+    </row>
+    <row r="99">
+      <c r="B99" t="s" s="1">
+        <v>695</v>
+      </c>
+      <c r="C99" t="s" s="1">
+        <v>696</v>
+      </c>
+      <c r="D99" t="s" s="1">
+        <v>697</v>
+      </c>
+      <c r="E99" t="s" s="1">
+        <v>698</v>
+      </c>
+      <c r="F99" t="s" s="1">
+        <v>699</v>
+      </c>
+      <c r="G99" t="s" s="1">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" t="s" s="1">
+        <v>701</v>
+      </c>
+      <c r="C100" t="s" s="1">
+        <v>702</v>
+      </c>
+      <c r="D100" s="1"/>
+      <c r="E100" t="b" s="1">
+        <v>1</v>
+      </c>
+      <c r="F100" t="s" s="1">
+        <v>703</v>
+      </c>
+      <c r="G100" t="s" s="1">
+        <v>704</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="77">
+  <mergeCells count="78">
     <mergeCell ref="D6:G6"/>
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="F10:G10"/>
@@ -7647,6 +7697,7 @@
     <mergeCell ref="D94:E94"/>
     <mergeCell ref="D95:E95"/>
     <mergeCell ref="D96:E96"/>
+    <mergeCell ref="B98:G98"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="J1" r:id="rId1" display="www.commerzbank.com"/>
@@ -7678,9 +7729,9 @@
   <dimension ref="B3:E25"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="31.66"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="27.11" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="27.44" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="0" width="31.66" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7867,9 +7918,9 @@
   <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="31.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="36"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="24.99" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="31.66" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="0" width="36.0" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8004,8 +8055,8 @@
   <dimension ref="C3:D13"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="25.66"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="22.66" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="25.66" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8098,18 +8149,18 @@
   <dimension ref="A1:O40"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="3.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="44.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="30.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="11.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="12.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="12.89"/>
+    <col min="1" max="1" customWidth="true" hidden="false" style="0" width="4.33" collapsed="false" outlineLevel="0"/>
+    <col min="2" max="2" customWidth="true" hidden="false" style="0" width="3.89" collapsed="false" outlineLevel="0"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="9.88" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="24.01" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="0" width="44.45" collapsed="false" outlineLevel="0"/>
+    <col min="6" max="6" customWidth="true" hidden="false" style="0" width="30.89" collapsed="false" outlineLevel="0"/>
+    <col min="7" max="7" customWidth="true" hidden="false" style="0" width="11.56" collapsed="false" outlineLevel="0"/>
+    <col min="8" max="8" customWidth="true" hidden="false" style="0" width="11.99" collapsed="false" outlineLevel="0"/>
+    <col min="9" max="9" customWidth="true" hidden="false" style="0" width="11.56" collapsed="false" outlineLevel="0"/>
+    <col min="10" max="10" customWidth="true" hidden="false" style="0" width="11.1" collapsed="false" outlineLevel="0"/>
+    <col min="11" max="12" customWidth="true" hidden="false" style="0" width="12.11" collapsed="false" outlineLevel="0"/>
+    <col min="13" max="13" customWidth="true" hidden="false" style="0" width="12.89" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8620,9 +8671,9 @@
   <dimension ref="C3:E9"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.34"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="20.66" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="30.56" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="0" width="19.34" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8700,11 +8751,11 @@
   <dimension ref="B1:F8"/>
   <sheetFormatPr defaultColWidth="9.09375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="95" width="9.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="95" width="18.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="95" width="13.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="95" width="14"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="6" style="95" width="9.11"/>
+    <col min="1" max="2" customWidth="false" hidden="false" style="95" width="9.11" collapsed="false" outlineLevel="0"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="95" width="18.22" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="95" width="13.56" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="95" width="14.0" collapsed="false" outlineLevel="0"/>
+    <col min="6" max="1024" customWidth="false" hidden="false" style="95" width="9.11" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8777,8 +8828,8 @@
   <dimension ref="B1:E21"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="76.22"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="28.44" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="76.22" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8946,8 +8997,8 @@
   <dimension ref="C3:D13"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26.11"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="20.44" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="26.11" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9020,10 +9071,10 @@
   <dimension ref="B2:E49"/>
   <sheetFormatPr defaultColWidth="9.09375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="95" width="9.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="95" width="17.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="95" width="39.11"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="5" style="95" width="9.11"/>
+    <col min="1" max="2" customWidth="false" hidden="false" style="95" width="9.11" collapsed="false" outlineLevel="0"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="95" width="17.67" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="95" width="39.11" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="1024" customWidth="false" hidden="false" style="95" width="9.11" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9448,10 +9499,10 @@
   <dimension ref="B3:D85"/>
   <sheetFormatPr defaultColWidth="9.09375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="1" style="95" width="9.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="95" width="34.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="95" width="29.99"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="6" style="95" width="9.11"/>
+    <col min="1" max="3" customWidth="false" hidden="false" style="95" width="9.11" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="95" width="34.44" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="95" width="29.99" collapsed="false" outlineLevel="0"/>
+    <col min="6" max="1024" customWidth="false" hidden="false" style="95" width="9.11" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9850,9 +9901,9 @@
   <dimension ref="A3:E43"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="38.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22.11"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="21.33" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="38.01" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="0" width="22.11" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10117,27 +10168,27 @@
   <dimension ref="B2:S90"/>
   <sheetFormatPr defaultColWidth="9.09375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="95" width="3.56"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="95" width="9.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="95" width="19.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="95" width="20.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="95" width="28.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="95" width="24.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="95" width="51.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="95" width="30.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="95" width="32.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="95" width="48.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="95" width="29.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="95" width="9.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="95" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="95" width="12.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="95" width="21.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="95" width="25.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="95" width="24.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="95" width="38.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="95" width="23.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="95" width="19.44"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="21" style="95" width="9.11"/>
+    <col min="1" max="1" customWidth="true" hidden="false" style="95" width="3.56" collapsed="false" outlineLevel="0"/>
+    <col min="2" max="2" customWidth="false" hidden="false" style="95" width="9.11" collapsed="false" outlineLevel="0"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="95" width="19.11" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="95" width="20.99" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="95" width="28.44" collapsed="false" outlineLevel="0"/>
+    <col min="6" max="6" customWidth="true" hidden="false" style="95" width="24.99" collapsed="false" outlineLevel="0"/>
+    <col min="7" max="7" customWidth="true" hidden="false" style="95" width="51.66" collapsed="false" outlineLevel="0"/>
+    <col min="8" max="8" customWidth="true" hidden="false" style="95" width="30.11" collapsed="false" outlineLevel="0"/>
+    <col min="9" max="9" customWidth="true" hidden="false" style="95" width="32.66" collapsed="false" outlineLevel="0"/>
+    <col min="10" max="10" customWidth="true" hidden="false" style="95" width="48.56" collapsed="false" outlineLevel="0"/>
+    <col min="11" max="11" customWidth="true" hidden="false" style="95" width="29.89" collapsed="false" outlineLevel="0"/>
+    <col min="12" max="12" customWidth="true" hidden="false" style="95" width="9.66" collapsed="false" outlineLevel="0"/>
+    <col min="13" max="13" customWidth="true" hidden="false" style="95" width="10.0" collapsed="false" outlineLevel="0"/>
+    <col min="14" max="14" customWidth="true" hidden="false" style="95" width="12.45" collapsed="false" outlineLevel="0"/>
+    <col min="15" max="15" customWidth="true" hidden="false" style="95" width="21.67" collapsed="false" outlineLevel="0"/>
+    <col min="16" max="16" customWidth="true" hidden="false" style="95" width="25.89" collapsed="false" outlineLevel="0"/>
+    <col min="17" max="17" customWidth="true" hidden="false" style="95" width="24.99" collapsed="false" outlineLevel="0"/>
+    <col min="18" max="18" customWidth="true" hidden="false" style="95" width="38.66" collapsed="false" outlineLevel="0"/>
+    <col min="19" max="19" customWidth="true" hidden="false" style="95" width="23.11" collapsed="false" outlineLevel="0"/>
+    <col min="20" max="20" customWidth="true" hidden="false" style="95" width="19.44" collapsed="false" outlineLevel="0"/>
+    <col min="21" max="1024" customWidth="false" hidden="false" style="95" width="9.11" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11354,10 +11405,10 @@
   <dimension ref="A1:I116"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="43.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9.88"/>
+    <col min="1" max="1" customWidth="true" hidden="false" style="0" width="9.11" collapsed="false" outlineLevel="0"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="43.56" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="34.32" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="0" width="9.88" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12070,10 +12121,10 @@
   <dimension ref="B3:D12"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="27.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24.56"/>
+    <col min="2" max="2" customWidth="true" hidden="false" style="0" width="14.11" collapsed="false" outlineLevel="0"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="23.11" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="27.11" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="0" width="24.56" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12159,9 +12210,9 @@
   <dimension ref="A3:J42"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="29.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="31.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26.33"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="29.99" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="31.66" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="0" width="26.33" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12441,9 +12492,9 @@
   <dimension ref="B3:E12"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="23.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="14.88" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="23.11" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="0" width="22.0" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12549,8 +12600,8 @@
   <dimension ref="A1:K58"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="31.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22.11"/>
+    <col min="3" max="4" customWidth="true" hidden="false" style="0" width="31.33" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="0" width="22.11" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12884,9 +12935,9 @@
   <dimension ref="B3:I20"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21.67"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="18.88" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="22.33" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="0" width="21.67" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13032,12 +13083,12 @@
   <dimension ref="A1:H41"/>
   <sheetFormatPr defaultColWidth="8.734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="35.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="26.33"/>
+    <col min="1" max="1" customWidth="true" hidden="false" style="0" width="9.11" collapsed="false" outlineLevel="0"/>
+    <col min="3" max="3" customWidth="true" hidden="false" style="0" width="44.89" collapsed="false" outlineLevel="0"/>
+    <col min="4" max="4" customWidth="true" hidden="false" style="0" width="40.44" collapsed="false" outlineLevel="0"/>
+    <col min="5" max="5" customWidth="true" hidden="false" style="0" width="35.33" collapsed="false" outlineLevel="0"/>
+    <col min="6" max="6" customWidth="true" hidden="false" style="0" width="15.1" collapsed="false" outlineLevel="0"/>
+    <col min="8" max="8" customWidth="true" hidden="false" style="0" width="26.33" collapsed="false" outlineLevel="0"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>